<commit_message>
Some work on Ghidra disassembly of TITLEPRG
</commit_message>
<xml_diff>
--- a/gamesource/church/Docs/Channel_XX_Structure.xlsx
+++ b/gamesource/church/Docs/Channel_XX_Structure.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\SourceCode\Amiga\Batman---Amiga\gamesource\church\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BF534DE-671E-4AF5-8582-97DCDEC96552}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA9E5B8C-66A5-4C0E-BC8D-2673F5113040}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="13770" activeTab="1" xr2:uid="{D9FDA9DF-FE4A-4B7C-BD85-712F15D68EFE}"/>
+    <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="13770" xr2:uid="{D9FDA9DF-FE4A-4B7C-BD85-712F15D68EFE}"/>
   </bookViews>
   <sheets>
     <sheet name="CHAN XX Struct" sheetId="1" r:id="rId1"/>

</xml_diff>